<commit_message>
First version of Localization Test Cases + Implementation
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Non-Functional Testing Suite/Localization  Tests.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Non-Functional Testing Suite/Localization  Tests.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -48,25 +48,108 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>1.</t>
-  </si>
-  <si>
-    <t>2.</t>
-  </si>
-  <si>
-    <t>3.</t>
+    <t>TC-L-1</t>
+  </si>
+  <si>
+    <t>Changing Language</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>1. Enter main Amazon web site  2. Enter the Sign In page</t>
+  </si>
+  <si>
+    <t>Verification of posibility to change the language form English to others</t>
+  </si>
+  <si>
+    <t>2. Tap on new chosen language</t>
+  </si>
+  <si>
+    <t>3. Save changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes of all text from the web application to the new language. </t>
+  </si>
+  <si>
+    <t>Status (Mobile)</t>
+  </si>
+  <si>
+    <t>Not Run</t>
+  </si>
+  <si>
+    <t>TC-L-2</t>
+  </si>
+  <si>
+    <t>For PC web applicatioon is possible to end up changing just by tapping on a menu that appears after pointing to the EN sign</t>
+  </si>
+  <si>
+    <t>1. Tap to EN (English) sign</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>TC-L-3</t>
+  </si>
+  <si>
+    <t>TC-L-4</t>
+  </si>
+  <si>
+    <t>TC-L-5</t>
+  </si>
+  <si>
+    <t>TC-L-6</t>
+  </si>
+  <si>
+    <t>Changing Money Currency</t>
+  </si>
+  <si>
+    <t>TC-L-7</t>
+  </si>
+  <si>
+    <t>Volume Measurement</t>
+  </si>
+  <si>
+    <t>Date Formatting</t>
+  </si>
+  <si>
+    <t>Time Formating</t>
+  </si>
+  <si>
+    <t>Length Formating</t>
+  </si>
+  <si>
+    <t>Weight Formating</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -142,22 +225,56 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -438,99 +555,618 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:J5"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" customWidth="1"/>
-    <col min="9" max="9" width="6.6640625" customWidth="1"/>
-    <col min="10" max="10" width="10.109375" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" customWidth="1"/>
+    <col min="5" max="5" width="30.109375" customWidth="1"/>
+    <col min="6" max="6" width="26.88671875" customWidth="1"/>
+    <col min="7" max="7" width="28.6640625" customWidth="1"/>
+    <col min="8" max="8" width="8" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
+    <col min="10" max="10" width="34.77734375" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" customWidth="1"/>
+    <col min="14" max="14" width="37.44140625" customWidth="1"/>
+    <col min="15" max="15" width="25.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="7"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+    </row>
+    <row r="3" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="11"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+      <c r="J3" s="11"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="12"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="12"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="7"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K8" s="7"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K9" s="7"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K10" s="7"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K11" s="7"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K12" s="7"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="1"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J20" s="1"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="5"/>
+      <c r="Q22" s="5"/>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23" s="6"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+      <c r="P23" s="5"/>
+      <c r="Q23" s="5"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="6"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="5"/>
+      <c r="O26" s="5"/>
+      <c r="P26" s="5"/>
+      <c r="Q26" s="5"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="5"/>
+      <c r="O27" s="5"/>
+      <c r="P27" s="5"/>
+      <c r="Q27" s="5"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
+      <c r="Q28" s="5"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" s="6"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="H3:H5"/>
+  <mergeCells count="63">
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="J29:J31"/>
+    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="D29:D31"/>
+    <mergeCell ref="E29:E31"/>
+    <mergeCell ref="G29:G31"/>
+    <mergeCell ref="H23:H25"/>
+    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="J23:J25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="E26:E28"/>
+    <mergeCell ref="G26:G28"/>
+    <mergeCell ref="H26:H28"/>
+    <mergeCell ref="I26:I28"/>
+    <mergeCell ref="J26:J28"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="G23:G25"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="J17:J19"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C20:C22"/>
+    <mergeCell ref="D20:D22"/>
+    <mergeCell ref="E20:E22"/>
+    <mergeCell ref="G20:G22"/>
+    <mergeCell ref="H20:H22"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="J20:J22"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="C17:C19"/>
+    <mergeCell ref="D17:D19"/>
+    <mergeCell ref="E17:E19"/>
+    <mergeCell ref="G17:G19"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="J2:J4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="I2:I4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="G2:G4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>